<commit_message>
Minor tinkering with plot creations, looking at eq_abundance without species interactions
</commit_message>
<xml_diff>
--- a/data/qPCR_Anatoxins_forGoel.xlsx
+++ b/data/qPCR_Anatoxins_forGoel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jld/Documents/Github/River_HAB_Modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B82EB483-6703-F442-A06F-0751D5B200A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B579148-FDFE-2E42-9181-F05316051307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="960" yWindow="1600" windowWidth="27640" windowHeight="16940" xr2:uid="{EF90CB1A-CFB2-4A4B-95FD-9B0D7CA467ED}"/>
   </bookViews>
@@ -137,9 +137,6 @@
     <t>bdl</t>
   </si>
   <si>
-    <t>Original file said 6.38 for ana_C/uL, but newer file from 1/2026 says NA</t>
-  </si>
-  <si>
     <t>Original file said 5404 for ana_C/ul, but newer file from 1/2026 says 43.9</t>
   </si>
   <si>
@@ -156,6 +153,9 @@
   </si>
   <si>
     <t>For ATXs in 2024, duplicates were averaged, and EXT samples were averaged</t>
+  </si>
+  <si>
+    <t>Original file (insert date) said 6.38 for ana_C/uL, but newer file from 1/2026 says NA</t>
   </si>
 </sst>
 </file>
@@ -650,14 +650,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1655,7 +1652,7 @@
       <c r="F22">
         <v>8</v>
       </c>
-      <c r="H22" s="3">
+      <c r="H22">
         <v>78</v>
       </c>
       <c r="J22">
@@ -2989,32 +2986,32 @@
         <v>2.5353500000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="4">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A55" s="1">
         <v>45181</v>
       </c>
-      <c r="B55" s="3">
-        <v>2023</v>
-      </c>
-      <c r="C55" s="3">
+      <c r="B55">
+        <v>2023</v>
+      </c>
+      <c r="C55">
         <v>2</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F55" s="3">
+      <c r="D55" t="s">
+        <v>18</v>
+      </c>
+      <c r="E55" t="s">
+        <v>19</v>
+      </c>
+      <c r="F55">
         <v>41</v>
       </c>
-      <c r="G55" s="3">
+      <c r="G55">
         <v>159</v>
       </c>
-      <c r="H55" s="3">
+      <c r="H55">
         <v>115</v>
       </c>
-      <c r="I55" s="3">
+      <c r="I55">
         <v>114.2</v>
       </c>
       <c r="J55" s="2">
@@ -3023,82 +3020,82 @@
       <c r="K55" s="2">
         <v>6388</v>
       </c>
-      <c r="L55" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M55" s="3">
-        <v>0</v>
-      </c>
-      <c r="N55" s="3">
+      <c r="L55" t="s">
+        <v>20</v>
+      </c>
+      <c r="M55">
+        <v>0</v>
+      </c>
+      <c r="N55">
         <v>9.8970000000000002</v>
       </c>
-      <c r="O55" s="3">
+      <c r="O55">
         <v>8.9819999999999993</v>
       </c>
-      <c r="P55" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q55" s="3">
+      <c r="P55" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q55">
         <v>0.91500000000000004</v>
       </c>
-      <c r="S55" s="3" t="s">
+      <c r="S55" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A56" s="1">
+        <v>45181</v>
+      </c>
+      <c r="B56">
+        <v>2023</v>
+      </c>
+      <c r="C56">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
+        <v>18</v>
+      </c>
+      <c r="E56" t="s">
+        <v>19</v>
+      </c>
+      <c r="F56">
+        <v>40</v>
+      </c>
+      <c r="G56">
+        <v>158</v>
+      </c>
+      <c r="H56">
+        <v>43</v>
+      </c>
+      <c r="I56">
+        <v>105.5</v>
+      </c>
+      <c r="J56">
+        <v>5404</v>
+      </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
+      <c r="L56" t="s">
+        <v>20</v>
+      </c>
+      <c r="M56">
+        <v>0</v>
+      </c>
+      <c r="N56">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="O56">
+        <v>18.323</v>
+      </c>
+      <c r="P56" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q56">
+        <v>1.667</v>
+      </c>
+      <c r="S56" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="4">
-        <v>45181</v>
-      </c>
-      <c r="B56" s="3">
-        <v>2023</v>
-      </c>
-      <c r="C56" s="3">
-        <v>3</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F56" s="3">
-        <v>40</v>
-      </c>
-      <c r="G56" s="3">
-        <v>158</v>
-      </c>
-      <c r="H56" s="3">
-        <v>43</v>
-      </c>
-      <c r="I56" s="3">
-        <v>105.5</v>
-      </c>
-      <c r="J56" s="3">
-        <v>5404</v>
-      </c>
-      <c r="K56" s="3">
-        <v>0</v>
-      </c>
-      <c r="L56" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M56" s="3">
-        <v>0</v>
-      </c>
-      <c r="N56" s="3">
-        <v>19.989999999999998</v>
-      </c>
-      <c r="O56" s="3">
-        <v>18.323</v>
-      </c>
-      <c r="P56" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q56" s="3">
-        <v>1.667</v>
-      </c>
-      <c r="S56" s="3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.2">
@@ -3453,10 +3450,10 @@
       <c r="I63">
         <v>130</v>
       </c>
-      <c r="J63">
+      <c r="J63" s="2">
         <v>41816</v>
       </c>
-      <c r="K63">
+      <c r="K63" s="2">
         <v>3870</v>
       </c>
       <c r="L63" t="s">
@@ -5445,7 +5442,7 @@
         <v>21</v>
       </c>
       <c r="S115" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="116" spans="1:19" x14ac:dyDescent="0.2">
@@ -5588,7 +5585,7 @@
         <v>33</v>
       </c>
       <c r="S119" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="120" spans="1:19" x14ac:dyDescent="0.2">
@@ -5799,7 +5796,7 @@
         <v>33</v>
       </c>
       <c r="S124" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="125" spans="1:19" x14ac:dyDescent="0.2">
@@ -5834,7 +5831,7 @@
         <v>30</v>
       </c>
       <c r="S125" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="126" spans="1:19" x14ac:dyDescent="0.2">
@@ -5919,7 +5916,7 @@
         <v>5.2999999999999999E-2</v>
       </c>
       <c r="S127" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="128" spans="1:19" x14ac:dyDescent="0.2">
@@ -6039,7 +6036,7 @@
         <v>0</v>
       </c>
       <c r="S130" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="131" spans="1:19" x14ac:dyDescent="0.2">
@@ -6070,20 +6067,20 @@
       <c r="L131">
         <v>46.6</v>
       </c>
-      <c r="N131" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="O131" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="P131" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q131" s="5" t="s">
+      <c r="N131" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O131" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P131" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q131" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S131" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="132" spans="1:19" x14ac:dyDescent="0.2">
@@ -6114,20 +6111,20 @@
       <c r="L132">
         <v>0</v>
       </c>
-      <c r="N132" s="6">
+      <c r="N132" s="3">
         <v>0.38</v>
       </c>
-      <c r="O132" s="6">
+      <c r="O132" s="3">
         <v>0.60200000000000009</v>
       </c>
-      <c r="P132" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q132" s="3">
+      <c r="P132" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q132">
         <v>9.9500000000000005E-2</v>
       </c>
       <c r="S132" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="133" spans="1:19" x14ac:dyDescent="0.2">
@@ -6281,20 +6278,20 @@
       <c r="L136">
         <v>0</v>
       </c>
-      <c r="N136" s="6">
+      <c r="N136" s="3">
         <v>2.5140000000000002</v>
       </c>
-      <c r="O136" s="6">
+      <c r="O136" s="3">
         <v>1.9824999999999999</v>
       </c>
-      <c r="P136" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q136" s="3">
+      <c r="P136" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q136">
         <v>0.53200000000000003</v>
       </c>
       <c r="S136" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="137" spans="1:19" x14ac:dyDescent="0.2">
@@ -6489,20 +6486,20 @@
       <c r="L141">
         <v>209</v>
       </c>
-      <c r="N141" s="5">
+      <c r="N141" s="3">
         <v>3.266666666666667E-2</v>
       </c>
-      <c r="O141" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="P141" s="5" t="s">
+      <c r="O141" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P141" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Q141">
         <v>3.266666666666667E-2</v>
       </c>
       <c r="S141" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="142" spans="1:19" x14ac:dyDescent="0.2">
@@ -6860,7 +6857,7 @@
         <v>33</v>
       </c>
       <c r="S152" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="153" spans="1:19" x14ac:dyDescent="0.2">
@@ -7060,7 +7057,7 @@
         <v>0</v>
       </c>
       <c r="S159" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="160" spans="1:19" x14ac:dyDescent="0.2">
@@ -7091,20 +7088,20 @@
       <c r="L160">
         <v>34938</v>
       </c>
-      <c r="N160" s="5">
+      <c r="N160" s="3">
         <v>1.1113333333333333</v>
       </c>
-      <c r="O160" s="5">
+      <c r="O160" s="3">
         <v>0.89833333333333332</v>
       </c>
-      <c r="P160" s="5" t="s">
+      <c r="P160" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Q160">
         <v>0.21366666666666667</v>
       </c>
       <c r="S160" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="161" spans="1:19" x14ac:dyDescent="0.2">
@@ -7135,20 +7132,20 @@
       <c r="L161">
         <v>1196</v>
       </c>
-      <c r="N161" s="6">
+      <c r="N161" s="3">
         <v>3.0274999999999999</v>
       </c>
-      <c r="O161" s="6">
+      <c r="O161" s="3">
         <v>2.71</v>
       </c>
-      <c r="P161" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q161" s="3">
+      <c r="P161" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q161">
         <v>0.3175</v>
       </c>
       <c r="S161" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="162" spans="1:19" x14ac:dyDescent="0.2">
@@ -7308,20 +7305,20 @@
       <c r="M165">
         <v>652</v>
       </c>
-      <c r="N165" s="5">
+      <c r="N165" s="3">
         <v>0.53799999999999992</v>
       </c>
-      <c r="O165" s="5">
+      <c r="O165" s="3">
         <v>0.44833333333333331</v>
       </c>
-      <c r="P165" s="5" t="s">
+      <c r="P165" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Q165">
         <v>8.9666666666666672E-2</v>
       </c>
       <c r="S165" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="166" spans="1:19" x14ac:dyDescent="0.2">
@@ -7393,20 +7390,20 @@
       <c r="L167">
         <v>1202</v>
       </c>
-      <c r="N167" s="5">
+      <c r="N167" s="3">
         <v>6.5780000000000003</v>
       </c>
-      <c r="O167" s="5">
+      <c r="O167" s="3">
         <v>4.7316666666666665</v>
       </c>
-      <c r="P167" s="5" t="s">
+      <c r="P167" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Q167">
         <v>1.8460000000000001</v>
       </c>
       <c r="S167" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="168" spans="1:19" x14ac:dyDescent="0.2">
@@ -7483,20 +7480,20 @@
       <c r="E170" t="s">
         <v>21</v>
       </c>
-      <c r="N170" s="5">
+      <c r="N170" s="3">
         <v>7.2333333333333319E-2</v>
       </c>
-      <c r="O170" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="P170" s="5" t="s">
+      <c r="O170" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P170" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Q170">
         <v>7.2333333333333319E-2</v>
       </c>
       <c r="S170" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="171" spans="1:19" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated and cleaned spreadsheets, added metadata direction into _forGoel file. Normalized ATX values with AFDM, and split sensitivity analysis into species included and excluded models
</commit_message>
<xml_diff>
--- a/data/qPCR_Anatoxins_forGoel.xlsx
+++ b/data/qPCR_Anatoxins_forGoel.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jld/Documents/Github/River_HAB_Modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B579148-FDFE-2E42-9181-F05316051307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB37516-E68D-AF47-B906-2CF2A7686525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="1600" windowWidth="27640" windowHeight="16940" xr2:uid="{EF90CB1A-CFB2-4A4B-95FD-9B0D7CA467ED}"/>
+    <workbookView xWindow="1600" yWindow="760" windowWidth="27640" windowHeight="18880" activeTab="1" xr2:uid="{EF90CB1A-CFB2-4A4B-95FD-9B0D7CA467ED}"/>
   </bookViews>
   <sheets>
     <sheet name="qPCR_Anatoxins" sheetId="1" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="74">
   <si>
     <t>date</t>
   </si>
@@ -155,14 +156,113 @@
     <t>For ATXs in 2024, duplicates were averaged, and EXT samples were averaged</t>
   </si>
   <si>
-    <t>Original file (insert date) said 6.38 for ana_C/uL, but newer file from 1/2026 says NA</t>
+    <t>org_matter_percent</t>
+  </si>
+  <si>
+    <t>Original file said 6.38 for ana_C/uL, but newer file from 1/2026 says NA</t>
+  </si>
+  <si>
+    <t>qPCR_Anatoxins.xlsx  Metadata</t>
+  </si>
+  <si>
+    <t>Column name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Date of sample collection</t>
+  </si>
+  <si>
+    <t>Reach names</t>
+  </si>
+  <si>
+    <t>This Excel file contains information about the number of ana_C and nif gene copies, as well as three anatoxin congener concentrations, found in Microcoleus and Anabaena mats. Percent organic material of each collected sample was calculated using ash-free dry mass weights. Gene copy values were extracted using qPCR methodology. Samples were collected from the South Fork Eel River in 2023 and 2024.</t>
+  </si>
+  <si>
+    <t>Year of sample collection</t>
+  </si>
+  <si>
+    <t>Old names vs. new names:</t>
+  </si>
+  <si>
+    <t>1S = 4S</t>
+  </si>
+  <si>
+    <t>2 = BUG</t>
+  </si>
+  <si>
+    <t>3 = 3UP</t>
+  </si>
+  <si>
+    <t>4 = 2UP</t>
+  </si>
+  <si>
+    <t>Genus of collected mat sample</t>
+  </si>
+  <si>
+    <t>Indicates whether mat material for qPCR analysis was present for collection in the field</t>
+  </si>
+  <si>
+    <t>sample_rerun</t>
+  </si>
+  <si>
+    <t>Vial ID # of samples (mailed in Oct. 2025)</t>
+  </si>
+  <si>
+    <t>DNA concentration in 250 mg of mat sample (vials mailed 2023)</t>
+  </si>
+  <si>
+    <t>Vial ID # of samples (mailed in 2023)</t>
+  </si>
+  <si>
+    <t>DNA concentration in 250 mg of mat sample (vials mailed 2025)</t>
+  </si>
+  <si>
+    <t>number of ana_C copies found per uL (vials mailed 2023)</t>
+  </si>
+  <si>
+    <t>number of ana_C copies found per uL (vials mailed 2025)</t>
+  </si>
+  <si>
+    <t>number of nif copies found per uL (vials mailed 2023)</t>
+  </si>
+  <si>
+    <t>number of nif copies found per uL (vials mailed 2025)</t>
+  </si>
+  <si>
+    <t>organic_matter_percent</t>
+  </si>
+  <si>
+    <t>Percent of organic matter found in each sample</t>
+  </si>
+  <si>
+    <t>Extra info supplied by UofU</t>
+  </si>
+  <si>
+    <t>Extra info supplied by UNR</t>
+  </si>
+  <si>
+    <t>Abbreviations</t>
+  </si>
+  <si>
+    <t>A collected sample was not analyzed (usually due to bad quality or insufficient volume)</t>
+  </si>
+  <si>
+    <t>Below detection limit. For anatoxins, unique detection limits were calculated per sample. Anatoxin detection limits not included in this file</t>
+  </si>
+  <si>
+    <t>Blank cell</t>
+  </si>
+  <si>
+    <t>No collected sample</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -300,7 +400,13 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="34">
@@ -650,11 +756,40 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1030,7 +1165,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA4CAA07-9486-4548-BA57-E25BF6238077}">
-  <dimension ref="A1:S173"/>
+  <dimension ref="A1:T173"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
@@ -1039,7 +1174,7 @@
     <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1092,13 +1227,16 @@
         <v>16</v>
       </c>
       <c r="R1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>45097</v>
       </c>
@@ -1127,7 +1265,7 @@
         <v>13807</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>45097</v>
       </c>
@@ -1144,7 +1282,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>45097</v>
       </c>
@@ -1161,7 +1299,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>45097</v>
       </c>
@@ -1178,7 +1316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>45102</v>
       </c>
@@ -1195,7 +1333,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>45102</v>
       </c>
@@ -1212,7 +1350,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>45102</v>
       </c>
@@ -1241,7 +1379,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>45102</v>
       </c>
@@ -1270,7 +1408,7 @@
         <v>3453</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>45110</v>
       </c>
@@ -1287,7 +1425,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>45110</v>
       </c>
@@ -1327,8 +1465,11 @@
       <c r="Q11" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R11">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>45110</v>
       </c>
@@ -1345,7 +1486,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>45110</v>
       </c>
@@ -1374,7 +1515,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>45117</v>
       </c>
@@ -1411,11 +1552,14 @@
       <c r="Q14" t="s">
         <v>33</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14">
+        <v>0.06</v>
+      </c>
+      <c r="S14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>45117</v>
       </c>
@@ -1455,8 +1599,11 @@
       <c r="Q15" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R15">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>45117</v>
       </c>
@@ -1473,7 +1620,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>45117</v>
       </c>
@@ -1513,8 +1660,11 @@
       <c r="Q17" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R17">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>45124</v>
       </c>
@@ -1531,7 +1681,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>45124</v>
       </c>
@@ -1571,8 +1721,11 @@
       <c r="Q19" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R19">
+        <v>0.69899999999999995</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>45124</v>
       </c>
@@ -1589,7 +1742,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>45124</v>
       </c>
@@ -1629,11 +1782,14 @@
       <c r="Q21" t="s">
         <v>33</v>
       </c>
-      <c r="R21" t="s">
+      <c r="R21">
+        <v>0.71</v>
+      </c>
+      <c r="S21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>45131</v>
       </c>
@@ -1673,8 +1829,11 @@
       <c r="Q22" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R22">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>45131</v>
       </c>
@@ -1714,8 +1873,11 @@
       <c r="Q23" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R23">
+        <v>0.628</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>45131</v>
       </c>
@@ -1744,7 +1906,7 @@
         <v>5096</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>45131</v>
       </c>
@@ -1784,8 +1946,11 @@
       <c r="Q25" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R25">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>45138</v>
       </c>
@@ -1807,11 +1972,11 @@
       <c r="I26">
         <v>75.3</v>
       </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-      <c r="M26">
-        <v>0</v>
+      <c r="K26" t="s">
+        <v>33</v>
+      </c>
+      <c r="M26" t="s">
+        <v>33</v>
       </c>
       <c r="N26">
         <v>8.1000000000000003E-2</v>
@@ -1825,8 +1990,11 @@
       <c r="Q26" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R26">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>45138</v>
       </c>
@@ -1857,14 +2025,14 @@
       <c r="J27" t="s">
         <v>20</v>
       </c>
-      <c r="K27">
-        <v>0</v>
+      <c r="K27" t="s">
+        <v>33</v>
       </c>
       <c r="L27" t="s">
         <v>20</v>
       </c>
-      <c r="M27">
-        <v>0</v>
+      <c r="M27" t="s">
+        <v>33</v>
       </c>
       <c r="N27">
         <v>0.313</v>
@@ -1878,8 +2046,11 @@
       <c r="Q27">
         <v>4.4999999999999998E-2</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R27">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>45138</v>
       </c>
@@ -1908,7 +2079,7 @@
         <v>3917</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>45138</v>
       </c>
@@ -1939,14 +2110,14 @@
       <c r="J29" t="s">
         <v>20</v>
       </c>
-      <c r="K29">
-        <v>0</v>
+      <c r="K29" t="s">
+        <v>33</v>
       </c>
       <c r="L29" t="s">
         <v>20</v>
       </c>
-      <c r="M29">
-        <v>0</v>
+      <c r="M29" t="s">
+        <v>33</v>
       </c>
       <c r="N29">
         <v>0.17799999999999999</v>
@@ -1960,8 +2131,11 @@
       <c r="Q29" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R29">
+        <v>0.70399999999999996</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>45145</v>
       </c>
@@ -1998,8 +2172,8 @@
       <c r="L30" t="s">
         <v>20</v>
       </c>
-      <c r="M30">
-        <v>0</v>
+      <c r="M30" t="s">
+        <v>33</v>
       </c>
       <c r="N30">
         <v>2.758</v>
@@ -2013,8 +2187,11 @@
       <c r="Q30">
         <v>0.33800000000000002</v>
       </c>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R30">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>45145</v>
       </c>
@@ -2045,14 +2222,14 @@
       <c r="J31" t="s">
         <v>20</v>
       </c>
-      <c r="K31">
-        <v>0</v>
+      <c r="K31" t="s">
+        <v>33</v>
       </c>
       <c r="L31" t="s">
         <v>20</v>
       </c>
-      <c r="M31">
-        <v>0</v>
+      <c r="M31" t="s">
+        <v>33</v>
       </c>
       <c r="N31">
         <v>1.8879999999999999</v>
@@ -2066,8 +2243,11 @@
       <c r="Q31">
         <v>0.35199999999999998</v>
       </c>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R31">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>45145</v>
       </c>
@@ -2107,8 +2287,11 @@
       <c r="Q32" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R32">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>45145</v>
       </c>
@@ -2139,14 +2322,14 @@
       <c r="J33" t="s">
         <v>20</v>
       </c>
-      <c r="K33">
-        <v>0</v>
+      <c r="K33" t="s">
+        <v>33</v>
       </c>
       <c r="L33" t="s">
         <v>20</v>
       </c>
-      <c r="M33">
-        <v>0</v>
+      <c r="M33" t="s">
+        <v>33</v>
       </c>
       <c r="N33">
         <v>0.36430000000000001</v>
@@ -2160,8 +2343,11 @@
       <c r="Q33">
         <v>7.0000000000000007E-2</v>
       </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R33">
+        <v>0.69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>45152</v>
       </c>
@@ -2186,8 +2372,8 @@
       <c r="J34">
         <v>141</v>
       </c>
-      <c r="L34">
-        <v>0</v>
+      <c r="L34" t="s">
+        <v>33</v>
       </c>
       <c r="N34">
         <v>1.9319999999999999</v>
@@ -2201,8 +2387,11 @@
       <c r="Q34">
         <v>0.28899999999999998</v>
       </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R34">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>45152</v>
       </c>
@@ -2233,14 +2422,14 @@
       <c r="J35" t="s">
         <v>20</v>
       </c>
-      <c r="K35">
-        <v>0</v>
+      <c r="K35" t="s">
+        <v>33</v>
       </c>
       <c r="L35" t="s">
         <v>20</v>
       </c>
-      <c r="M35">
-        <v>0</v>
+      <c r="M35" t="s">
+        <v>33</v>
       </c>
       <c r="N35">
         <v>6.6467000000000001</v>
@@ -2254,8 +2443,11 @@
       <c r="Q35">
         <v>1.1476999999999999</v>
       </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R35">
+        <v>0.751</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>45152</v>
       </c>
@@ -2284,7 +2476,7 @@
         <v>3047</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>45152</v>
       </c>
@@ -2312,8 +2504,8 @@
       <c r="I37" t="s">
         <v>20</v>
       </c>
-      <c r="J37">
-        <v>0</v>
+      <c r="J37" t="s">
+        <v>33</v>
       </c>
       <c r="K37" t="s">
         <v>20</v>
@@ -2336,11 +2528,14 @@
       <c r="Q37">
         <v>4.9500000000000002E-2</v>
       </c>
-      <c r="R37" t="s">
+      <c r="R37">
+        <v>0.75</v>
+      </c>
+      <c r="S37" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>45160</v>
       </c>
@@ -2365,8 +2560,8 @@
       <c r="J38">
         <v>3.37</v>
       </c>
-      <c r="L38">
-        <v>0</v>
+      <c r="L38" t="s">
+        <v>33</v>
       </c>
       <c r="N38">
         <v>17.29</v>
@@ -2380,8 +2575,11 @@
       <c r="Q38">
         <v>2.57</v>
       </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R38">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>45160</v>
       </c>
@@ -2412,14 +2610,14 @@
       <c r="J39" t="s">
         <v>20</v>
       </c>
-      <c r="K39">
-        <v>0</v>
+      <c r="K39" t="s">
+        <v>33</v>
       </c>
       <c r="L39" t="s">
         <v>20</v>
       </c>
-      <c r="M39">
-        <v>0</v>
+      <c r="M39" t="s">
+        <v>33</v>
       </c>
       <c r="N39">
         <v>7.3623000000000003</v>
@@ -2433,8 +2631,11 @@
       <c r="Q39">
         <v>1.071</v>
       </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R39">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>45160</v>
       </c>
@@ -2459,8 +2660,8 @@
       <c r="K40">
         <v>7161</v>
       </c>
-      <c r="M40">
-        <v>0</v>
+      <c r="M40" t="s">
+        <v>33</v>
       </c>
       <c r="N40">
         <v>99.066000000000003</v>
@@ -2474,8 +2675,11 @@
       <c r="Q40">
         <v>15.628</v>
       </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R40">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>45160</v>
       </c>
@@ -2527,11 +2731,14 @@
       <c r="Q41">
         <v>0.436</v>
       </c>
-      <c r="R41" t="s">
+      <c r="R41">
+        <v>0.68</v>
+      </c>
+      <c r="S41" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>45162</v>
       </c>
@@ -2553,17 +2760,17 @@
       <c r="H42">
         <v>49</v>
       </c>
-      <c r="J42">
-        <v>0</v>
-      </c>
-      <c r="L42">
-        <v>0</v>
-      </c>
-      <c r="S42" t="s">
+      <c r="J42" t="s">
+        <v>33</v>
+      </c>
+      <c r="L42" t="s">
+        <v>33</v>
+      </c>
+      <c r="T42" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>45162</v>
       </c>
@@ -2579,11 +2786,11 @@
       <c r="E43" t="s">
         <v>21</v>
       </c>
-      <c r="S43" t="s">
+      <c r="T43" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>45162</v>
       </c>
@@ -2599,11 +2806,11 @@
       <c r="E44" t="s">
         <v>21</v>
       </c>
-      <c r="S44" t="s">
+      <c r="T44" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>45162</v>
       </c>
@@ -2619,11 +2826,11 @@
       <c r="E45" t="s">
         <v>21</v>
       </c>
-      <c r="S45" t="s">
+      <c r="T45" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>45166</v>
       </c>
@@ -2651,8 +2858,8 @@
       <c r="I46">
         <v>68</v>
       </c>
-      <c r="J46">
-        <v>0</v>
+      <c r="J46" t="s">
+        <v>33</v>
       </c>
       <c r="K46">
         <v>4930</v>
@@ -2675,8 +2882,11 @@
       <c r="Q46">
         <v>2.5289999999999999</v>
       </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R46">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>45166</v>
       </c>
@@ -2698,17 +2908,17 @@
       <c r="H47">
         <v>19</v>
       </c>
-      <c r="J47">
-        <v>0</v>
-      </c>
-      <c r="L47">
-        <v>0</v>
-      </c>
-      <c r="S47" t="s">
+      <c r="J47" t="s">
+        <v>33</v>
+      </c>
+      <c r="L47" t="s">
+        <v>33</v>
+      </c>
+      <c r="T47" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>45166</v>
       </c>
@@ -2748,8 +2958,11 @@
       <c r="Q48">
         <v>3.198</v>
       </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R48">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>45166</v>
       </c>
@@ -2778,7 +2991,7 @@
         <v>78.3</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>45166</v>
       </c>
@@ -2818,8 +3031,11 @@
       <c r="Q50">
         <v>1.1611499999999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R50">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>45173</v>
       </c>
@@ -2844,8 +3060,8 @@
       <c r="J51">
         <v>85.1</v>
       </c>
-      <c r="L51">
-        <v>0</v>
+      <c r="L51" t="s">
+        <v>33</v>
       </c>
       <c r="N51">
         <v>18.032</v>
@@ -2859,8 +3075,11 @@
       <c r="Q51">
         <v>2.032</v>
       </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R51">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>45173</v>
       </c>
@@ -2885,8 +3104,8 @@
       <c r="J52">
         <v>43.9</v>
       </c>
-      <c r="L52">
-        <v>0</v>
+      <c r="L52" t="s">
+        <v>33</v>
       </c>
       <c r="N52">
         <v>25.83</v>
@@ -2900,8 +3119,11 @@
       <c r="Q52">
         <v>2.867</v>
       </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R52">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>45173</v>
       </c>
@@ -2941,11 +3163,14 @@
       <c r="Q53">
         <v>0.23799999999999999</v>
       </c>
-      <c r="R53" t="s">
+      <c r="R53">
+        <v>0.34</v>
+      </c>
+      <c r="S53" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>45173</v>
       </c>
@@ -2985,8 +3210,11 @@
       <c r="Q54">
         <v>2.5353500000000002</v>
       </c>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R54">
+        <v>0.75700000000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>45181</v>
       </c>
@@ -3023,8 +3251,8 @@
       <c r="L55" t="s">
         <v>20</v>
       </c>
-      <c r="M55">
-        <v>0</v>
+      <c r="M55" t="s">
+        <v>33</v>
       </c>
       <c r="N55">
         <v>9.8970000000000002</v>
@@ -3038,11 +3266,14 @@
       <c r="Q55">
         <v>0.91500000000000004</v>
       </c>
-      <c r="S55" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R55">
+        <v>0.61299999999999999</v>
+      </c>
+      <c r="T55" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>45181</v>
       </c>
@@ -3073,14 +3304,14 @@
       <c r="J56">
         <v>5404</v>
       </c>
-      <c r="K56">
-        <v>0</v>
+      <c r="K56" t="s">
+        <v>33</v>
       </c>
       <c r="L56" t="s">
         <v>20</v>
       </c>
-      <c r="M56">
-        <v>0</v>
+      <c r="M56" t="s">
+        <v>33</v>
       </c>
       <c r="N56">
         <v>19.989999999999998</v>
@@ -3094,11 +3325,14 @@
       <c r="Q56">
         <v>1.667</v>
       </c>
-      <c r="S56" t="s">
+      <c r="R56">
+        <v>0.73</v>
+      </c>
+      <c r="T56" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>45181</v>
       </c>
@@ -3126,8 +3360,8 @@
       <c r="I57">
         <v>57.3</v>
       </c>
-      <c r="J57" s="2">
-        <v>0</v>
+      <c r="J57" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="K57" s="2">
         <v>20904</v>
@@ -3150,8 +3384,11 @@
       <c r="Q57">
         <v>9.5000000000000001E-2</v>
       </c>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R57">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>45181</v>
       </c>
@@ -3203,11 +3440,14 @@
       <c r="Q58">
         <v>0.81950000000000001</v>
       </c>
-      <c r="R58" t="s">
+      <c r="R58">
+        <v>0.76</v>
+      </c>
+      <c r="S58" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>45187</v>
       </c>
@@ -3259,11 +3499,14 @@
       <c r="Q59">
         <v>0.45800000000000002</v>
       </c>
-      <c r="R59" t="s">
+      <c r="R59">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="S59" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>45187</v>
       </c>
@@ -3294,14 +3537,14 @@
       <c r="J60">
         <v>103</v>
       </c>
-      <c r="K60">
-        <v>0</v>
+      <c r="K60" t="s">
+        <v>33</v>
       </c>
       <c r="L60" t="s">
         <v>20</v>
       </c>
-      <c r="M60">
-        <v>0</v>
+      <c r="M60" t="s">
+        <v>33</v>
       </c>
       <c r="N60">
         <v>12.81</v>
@@ -3315,8 +3558,11 @@
       <c r="Q60">
         <v>1.1479999999999999</v>
       </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R60">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>45187</v>
       </c>
@@ -3344,8 +3590,8 @@
       <c r="I61">
         <v>96.1</v>
       </c>
-      <c r="J61" s="2">
-        <v>0</v>
+      <c r="J61" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="K61" s="2">
         <v>22269</v>
@@ -3368,8 +3614,11 @@
       <c r="Q61">
         <v>6.2E-2</v>
       </c>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R61">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>45187</v>
       </c>
@@ -3421,8 +3670,11 @@
       <c r="Q62">
         <v>2.9834999999999998</v>
       </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R62">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>45193</v>
       </c>
@@ -3450,10 +3702,10 @@
       <c r="I63">
         <v>130</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63">
         <v>41816</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63">
         <v>3870</v>
       </c>
       <c r="L63" t="s">
@@ -3474,8 +3726,11 @@
       <c r="Q63">
         <v>0.29570000000000002</v>
       </c>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R63">
+        <v>0.57599999999999996</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>45193</v>
       </c>
@@ -3527,11 +3782,14 @@
       <c r="Q64">
         <v>0.32600000000000001</v>
       </c>
-      <c r="R64" t="s">
+      <c r="R64">
+        <v>0.76</v>
+      </c>
+      <c r="S64" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>45193</v>
       </c>
@@ -3583,8 +3841,11 @@
       <c r="Q65" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R65">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>45193</v>
       </c>
@@ -3636,11 +3897,14 @@
       <c r="Q66">
         <v>1.04</v>
       </c>
-      <c r="R66" t="s">
+      <c r="R66">
+        <v>0.79</v>
+      </c>
+      <c r="S66" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>45117</v>
       </c>
@@ -3668,11 +3932,11 @@
       <c r="M67" t="s">
         <v>20</v>
       </c>
-      <c r="R67" t="s">
+      <c r="S67" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>45117</v>
       </c>
@@ -3700,11 +3964,11 @@
       <c r="M68" t="s">
         <v>20</v>
       </c>
-      <c r="R68" t="s">
+      <c r="S68" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>45117</v>
       </c>
@@ -3744,11 +4008,14 @@
       <c r="Q69" t="s">
         <v>33</v>
       </c>
-      <c r="R69" t="s">
+      <c r="R69">
+        <v>0.67</v>
+      </c>
+      <c r="S69" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>45117</v>
       </c>
@@ -3770,8 +4037,8 @@
       <c r="I70">
         <v>58.1</v>
       </c>
-      <c r="K70">
-        <v>0</v>
+      <c r="K70" t="s">
+        <v>33</v>
       </c>
       <c r="M70">
         <v>870</v>
@@ -3788,8 +4055,11 @@
       <c r="Q70" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R70">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>45124</v>
       </c>
@@ -3818,7 +4088,7 @@
         <v>6690</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>45124</v>
       </c>
@@ -3847,7 +4117,7 @@
         <v>17670</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>45124</v>
       </c>
@@ -3869,8 +4139,8 @@
       <c r="I73">
         <v>84.6</v>
       </c>
-      <c r="K73">
-        <v>0</v>
+      <c r="K73" t="s">
+        <v>33</v>
       </c>
       <c r="M73">
         <v>1299</v>
@@ -3887,8 +4157,11 @@
       <c r="Q73" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R73">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="74" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>45124</v>
       </c>
@@ -3928,8 +4201,11 @@
       <c r="Q74" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R74">
+        <v>0.54300000000000004</v>
+      </c>
+    </row>
+    <row r="75" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>45131</v>
       </c>
@@ -3969,8 +4245,11 @@
       <c r="Q75">
         <v>0.16500000000000001</v>
       </c>
-    </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R75">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>45131</v>
       </c>
@@ -3992,11 +4271,11 @@
       <c r="I76">
         <v>65.2</v>
       </c>
-      <c r="K76">
-        <v>0</v>
-      </c>
-      <c r="M76">
-        <v>0</v>
+      <c r="K76" t="s">
+        <v>33</v>
+      </c>
+      <c r="M76" t="s">
+        <v>33</v>
       </c>
       <c r="N76">
         <v>8.7999999999999995E-2</v>
@@ -4010,8 +4289,11 @@
       <c r="Q76">
         <v>6.2E-2</v>
       </c>
-    </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R76">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>45131</v>
       </c>
@@ -4033,11 +4315,11 @@
       <c r="I77">
         <v>59.9</v>
       </c>
-      <c r="K77">
-        <v>0</v>
-      </c>
-      <c r="M77">
-        <v>0</v>
+      <c r="K77" t="s">
+        <v>33</v>
+      </c>
+      <c r="M77" t="s">
+        <v>33</v>
       </c>
       <c r="N77">
         <v>0.77800000000000002</v>
@@ -4051,8 +4333,11 @@
       <c r="Q77">
         <v>0.17299999999999999</v>
       </c>
-    </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R77">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>45131</v>
       </c>
@@ -4080,8 +4365,11 @@
       <c r="Q78">
         <v>2.4500000000000001E-2</v>
       </c>
-    </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R78">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>45138</v>
       </c>
@@ -4103,11 +4391,11 @@
       <c r="I79">
         <v>159</v>
       </c>
-      <c r="K79">
-        <v>0</v>
-      </c>
-      <c r="M79">
-        <v>0</v>
+      <c r="K79" t="s">
+        <v>33</v>
+      </c>
+      <c r="M79" t="s">
+        <v>33</v>
       </c>
       <c r="N79">
         <v>5.0190000000000001</v>
@@ -4121,8 +4409,11 @@
       <c r="Q79">
         <v>0.79200000000000004</v>
       </c>
-    </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R79">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>45138</v>
       </c>
@@ -4144,11 +4435,11 @@
       <c r="I80">
         <v>80.7</v>
       </c>
-      <c r="K80">
-        <v>0</v>
-      </c>
-      <c r="M80">
-        <v>0</v>
+      <c r="K80" t="s">
+        <v>33</v>
+      </c>
+      <c r="M80" t="s">
+        <v>33</v>
       </c>
       <c r="N80">
         <v>0.76300000000000001</v>
@@ -4162,8 +4453,11 @@
       <c r="Q80">
         <v>0.17499999999999999</v>
       </c>
-    </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R80">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>45138</v>
       </c>
@@ -4203,11 +4497,14 @@
       <c r="Q81">
         <v>1.1259999999999999</v>
       </c>
-      <c r="R81" t="s">
+      <c r="R81">
+        <v>0.42</v>
+      </c>
+      <c r="S81" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>45138</v>
       </c>
@@ -4232,8 +4529,8 @@
       <c r="K82">
         <v>12.8</v>
       </c>
-      <c r="M82">
-        <v>0</v>
+      <c r="M82" t="s">
+        <v>33</v>
       </c>
       <c r="N82">
         <v>3.6920000000000002</v>
@@ -4247,8 +4544,11 @@
       <c r="Q82">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R82">
+        <v>0.41299999999999998</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>45145</v>
       </c>
@@ -4270,8 +4570,8 @@
       <c r="I83">
         <v>132</v>
       </c>
-      <c r="K83">
-        <v>0</v>
+      <c r="K83" t="s">
+        <v>33</v>
       </c>
       <c r="M83">
         <v>29532</v>
@@ -4288,8 +4588,11 @@
       <c r="Q83">
         <v>8.7999999999999995E-2</v>
       </c>
-    </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R83">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>45145</v>
       </c>
@@ -4329,8 +4632,11 @@
       <c r="Q84">
         <v>0.68300000000000005</v>
       </c>
-    </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R84">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>45145</v>
       </c>
@@ -4352,11 +4658,11 @@
       <c r="I85">
         <v>76.2</v>
       </c>
-      <c r="K85">
-        <v>0</v>
-      </c>
-      <c r="M85">
-        <v>0</v>
+      <c r="K85" t="s">
+        <v>33</v>
+      </c>
+      <c r="M85" t="s">
+        <v>33</v>
       </c>
       <c r="N85">
         <v>38.588000000000001</v>
@@ -4370,8 +4676,11 @@
       <c r="Q85">
         <v>4.34</v>
       </c>
-    </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R85">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>45145</v>
       </c>
@@ -4396,8 +4705,8 @@
       <c r="K86">
         <v>37339</v>
       </c>
-      <c r="M86">
-        <v>0</v>
+      <c r="M86" t="s">
+        <v>33</v>
       </c>
       <c r="N86">
         <v>7.1319999999999997</v>
@@ -4411,8 +4720,11 @@
       <c r="Q86">
         <v>0.75834999999999997</v>
       </c>
-    </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R86">
+        <v>0.38600000000000001</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>45152</v>
       </c>
@@ -4434,11 +4746,11 @@
       <c r="I87">
         <v>58.6</v>
       </c>
-      <c r="K87">
-        <v>0</v>
-      </c>
-      <c r="M87">
-        <v>0</v>
+      <c r="K87" t="s">
+        <v>33</v>
+      </c>
+      <c r="M87" t="s">
+        <v>33</v>
       </c>
       <c r="N87">
         <v>51.351999999999997</v>
@@ -4452,8 +4764,11 @@
       <c r="Q87">
         <v>5.6950000000000003</v>
       </c>
-    </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R87">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>45152</v>
       </c>
@@ -4478,8 +4793,8 @@
       <c r="K88">
         <v>16234</v>
       </c>
-      <c r="M88">
-        <v>0</v>
+      <c r="M88" t="s">
+        <v>33</v>
       </c>
       <c r="N88">
         <v>24.847300000000001</v>
@@ -4493,8 +4808,11 @@
       <c r="Q88">
         <v>3.0489999999999999</v>
       </c>
-    </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R88">
+        <v>0.56799999999999995</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>45152</v>
       </c>
@@ -4516,11 +4834,11 @@
       <c r="I89">
         <v>47.9</v>
       </c>
-      <c r="K89">
-        <v>0</v>
-      </c>
-      <c r="M89">
-        <v>0</v>
+      <c r="K89" t="s">
+        <v>33</v>
+      </c>
+      <c r="M89" t="s">
+        <v>33</v>
       </c>
       <c r="N89">
         <v>25.082000000000001</v>
@@ -4534,8 +4852,11 @@
       <c r="Q89">
         <v>3.6040000000000001</v>
       </c>
-    </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R89">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>45152</v>
       </c>
@@ -4557,11 +4878,11 @@
       <c r="I90">
         <v>188.1</v>
       </c>
-      <c r="K90">
-        <v>0</v>
-      </c>
-      <c r="M90">
-        <v>0</v>
+      <c r="K90" t="s">
+        <v>33</v>
+      </c>
+      <c r="M90" t="s">
+        <v>33</v>
       </c>
       <c r="N90">
         <v>36.5015</v>
@@ -4575,8 +4896,11 @@
       <c r="Q90">
         <v>4.2065000000000001</v>
       </c>
-    </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R90">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>45160</v>
       </c>
@@ -4616,8 +4940,11 @@
       <c r="Q91">
         <v>0.94199999999999995</v>
       </c>
-    </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R91">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>45160</v>
       </c>
@@ -4657,8 +4984,11 @@
       <c r="Q92">
         <v>3.1259999999999999</v>
       </c>
-    </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R92">
+        <v>0.434</v>
+      </c>
+    </row>
+    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>45160</v>
       </c>
@@ -4680,11 +5010,11 @@
       <c r="I93">
         <v>28.2</v>
       </c>
-      <c r="K93">
-        <v>0</v>
-      </c>
-      <c r="M93">
-        <v>0</v>
+      <c r="K93" t="s">
+        <v>33</v>
+      </c>
+      <c r="M93" t="s">
+        <v>33</v>
       </c>
       <c r="N93">
         <v>32.741</v>
@@ -4698,8 +5028,11 @@
       <c r="Q93">
         <v>3.9239999999999999</v>
       </c>
-    </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R93">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>45160</v>
       </c>
@@ -4721,11 +5054,11 @@
       <c r="I94">
         <v>151.80000000000001</v>
       </c>
-      <c r="K94">
-        <v>0</v>
-      </c>
-      <c r="M94">
-        <v>0</v>
+      <c r="K94" t="s">
+        <v>33</v>
+      </c>
+      <c r="M94" t="s">
+        <v>33</v>
       </c>
       <c r="N94">
         <v>15.971500000000001</v>
@@ -4739,8 +5072,11 @@
       <c r="Q94">
         <v>1.984</v>
       </c>
-    </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R94">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="95" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>45166</v>
       </c>
@@ -4768,11 +5104,11 @@
       <c r="M95" t="s">
         <v>20</v>
       </c>
-      <c r="R95" t="s">
+      <c r="S95" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>45166</v>
       </c>
@@ -4812,11 +5148,14 @@
       <c r="Q96">
         <v>0.153</v>
       </c>
-      <c r="R96" t="s">
+      <c r="R96">
+        <v>0.38</v>
+      </c>
+      <c r="S96" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>45166</v>
       </c>
@@ -4838,14 +5177,14 @@
       <c r="I97">
         <v>63.7</v>
       </c>
-      <c r="K97">
-        <v>0</v>
-      </c>
-      <c r="M97">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="K97" t="s">
+        <v>33</v>
+      </c>
+      <c r="M97" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="98" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>45166</v>
       </c>
@@ -4885,11 +5224,14 @@
       <c r="Q98">
         <v>1.9279999999999999</v>
       </c>
-      <c r="R98" t="s">
+      <c r="R98">
+        <v>1.2</v>
+      </c>
+      <c r="S98" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>45173</v>
       </c>
@@ -4929,8 +5271,11 @@
       <c r="Q99" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R99">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="100" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>45173</v>
       </c>
@@ -4958,11 +5303,11 @@
       <c r="M100" t="s">
         <v>20</v>
       </c>
-      <c r="R100" t="s">
+      <c r="S100" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>45173</v>
       </c>
@@ -4979,7 +5324,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>45173</v>
       </c>
@@ -5019,11 +5364,14 @@
       <c r="Q102">
         <v>0.29799999999999999</v>
       </c>
-      <c r="R102" t="s">
+      <c r="R102">
+        <v>0.44700000000000001</v>
+      </c>
+      <c r="S102" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>45181</v>
       </c>
@@ -5040,7 +5388,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>45181</v>
       </c>
@@ -5057,7 +5405,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
         <v>45181</v>
       </c>
@@ -5074,7 +5422,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
         <v>45181</v>
       </c>
@@ -5114,8 +5462,11 @@
       <c r="Q106" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R106">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
         <v>45187</v>
       </c>
@@ -5155,11 +5506,14 @@
       <c r="Q107" t="s">
         <v>33</v>
       </c>
-      <c r="R107" t="s">
+      <c r="R107">
+        <v>0.15</v>
+      </c>
+      <c r="S107" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
         <v>45187</v>
       </c>
@@ -5199,11 +5553,14 @@
       <c r="Q108" t="s">
         <v>33</v>
       </c>
-      <c r="R108" t="s">
+      <c r="R108">
+        <v>0.26300000000000001</v>
+      </c>
+      <c r="S108" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
         <v>45187</v>
       </c>
@@ -5232,7 +5589,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
         <v>45187</v>
       </c>
@@ -5272,11 +5629,14 @@
       <c r="Q110">
         <v>0.57950000000000002</v>
       </c>
-      <c r="R110" t="s">
+      <c r="R110">
+        <v>0.31</v>
+      </c>
+      <c r="S110" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
         <v>45193</v>
       </c>
@@ -5316,11 +5676,14 @@
       <c r="Q111" t="s">
         <v>33</v>
       </c>
-      <c r="R111" t="s">
+      <c r="R111">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="S111" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
         <v>45193</v>
       </c>
@@ -5348,11 +5711,11 @@
       <c r="M112" t="s">
         <v>20</v>
       </c>
-      <c r="R112" t="s">
+      <c r="S112" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
         <v>45193</v>
       </c>
@@ -5380,11 +5743,11 @@
       <c r="M113" t="s">
         <v>20</v>
       </c>
-      <c r="R113" t="s">
+      <c r="S113" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
         <v>45193</v>
       </c>
@@ -5424,8 +5787,11 @@
       <c r="Q114">
         <v>4.5499999999999999E-2</v>
       </c>
-    </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R114">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
         <v>45462</v>
       </c>
@@ -5441,11 +5807,11 @@
       <c r="E115" t="s">
         <v>21</v>
       </c>
-      <c r="S115" t="s">
+      <c r="T115" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
         <v>45462</v>
       </c>
@@ -5474,7 +5840,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
         <v>45462</v>
       </c>
@@ -5514,8 +5880,11 @@
       <c r="Q117" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R117">
+        <v>0.73529999999999995</v>
+      </c>
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
         <v>45462</v>
       </c>
@@ -5540,8 +5909,8 @@
       <c r="J118">
         <v>5.31</v>
       </c>
-      <c r="L118">
-        <v>0</v>
+      <c r="L118" t="s">
+        <v>33</v>
       </c>
       <c r="N118" t="s">
         <v>33</v>
@@ -5555,8 +5924,11 @@
       <c r="Q118" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R118">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
         <v>45475</v>
       </c>
@@ -5584,11 +5956,14 @@
       <c r="Q119" t="s">
         <v>33</v>
       </c>
-      <c r="S119" t="s">
+      <c r="R119">
+        <v>0.3528</v>
+      </c>
+      <c r="T119" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
         <v>45475</v>
       </c>
@@ -5610,11 +5985,11 @@
       <c r="H120">
         <v>384.8</v>
       </c>
-      <c r="J120">
-        <v>0</v>
-      </c>
-      <c r="L120">
-        <v>0</v>
+      <c r="J120" t="s">
+        <v>33</v>
+      </c>
+      <c r="L120" t="s">
+        <v>33</v>
       </c>
       <c r="N120" t="s">
         <v>33</v>
@@ -5628,8 +6003,11 @@
       <c r="Q120" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R120">
+        <v>0.60550000000000004</v>
+      </c>
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
         <v>45475</v>
       </c>
@@ -5669,8 +6047,11 @@
       <c r="Q121" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R121">
+        <v>0.60450000000000004</v>
+      </c>
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
         <v>45475</v>
       </c>
@@ -5692,8 +6073,8 @@
       <c r="H122">
         <v>60.3</v>
       </c>
-      <c r="J122">
-        <v>0</v>
+      <c r="J122" t="s">
+        <v>33</v>
       </c>
       <c r="L122">
         <v>17562</v>
@@ -5710,8 +6091,11 @@
       <c r="Q122" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R122">
+        <v>0.59289999999999998</v>
+      </c>
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
         <v>45490</v>
       </c>
@@ -5751,8 +6135,11 @@
       <c r="Q123" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R123">
+        <v>0.39500000000000002</v>
+      </c>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
         <v>45490</v>
       </c>
@@ -5780,8 +6167,8 @@
       <c r="K124">
         <v>271</v>
       </c>
-      <c r="L124">
-        <v>0</v>
+      <c r="L124" t="s">
+        <v>33</v>
       </c>
       <c r="N124" t="s">
         <v>33</v>
@@ -5795,11 +6182,14 @@
       <c r="Q124" t="s">
         <v>33</v>
       </c>
-      <c r="S124" t="s">
+      <c r="R124">
+        <v>0.6139</v>
+      </c>
+      <c r="T124" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
         <v>45490</v>
       </c>
@@ -5830,11 +6220,26 @@
       <c r="L125">
         <v>30</v>
       </c>
-      <c r="S125" t="s">
+      <c r="N125" t="s">
+        <v>33</v>
+      </c>
+      <c r="O125" t="s">
+        <v>33</v>
+      </c>
+      <c r="P125" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q125" t="s">
+        <v>33</v>
+      </c>
+      <c r="R125">
+        <v>0.6139</v>
+      </c>
+      <c r="T125" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
         <v>45490</v>
       </c>
@@ -5859,8 +6264,8 @@
       <c r="J126">
         <v>22.1</v>
       </c>
-      <c r="L126">
-        <v>0</v>
+      <c r="L126" t="s">
+        <v>33</v>
       </c>
       <c r="N126" t="s">
         <v>33</v>
@@ -5874,8 +6279,11 @@
       <c r="Q126" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R126">
+        <v>9.6299999999999997E-2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
         <v>45490</v>
       </c>
@@ -5915,11 +6323,14 @@
       <c r="Q127">
         <v>5.2999999999999999E-2</v>
       </c>
-      <c r="S127" t="s">
+      <c r="R127">
+        <v>0.56040000000000001</v>
+      </c>
+      <c r="T127" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
         <v>45504</v>
       </c>
@@ -5959,8 +6370,11 @@
       <c r="Q128" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R128">
+        <v>9.8100000000000007E-2</v>
+      </c>
+    </row>
+    <row r="129" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A129" s="1">
         <v>45504</v>
       </c>
@@ -5982,14 +6396,14 @@
       <c r="H129">
         <v>347</v>
       </c>
-      <c r="J129">
-        <v>0</v>
+      <c r="J129" t="s">
+        <v>33</v>
       </c>
       <c r="K129">
         <v>10.67</v>
       </c>
-      <c r="L129">
-        <v>0</v>
+      <c r="L129" t="s">
+        <v>33</v>
       </c>
       <c r="N129">
         <v>5.8999999999999997E-2</v>
@@ -6003,8 +6417,11 @@
       <c r="Q129">
         <v>5.8999999999999997E-2</v>
       </c>
-    </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R129">
+        <v>0.75990000000000002</v>
+      </c>
+    </row>
+    <row r="130" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
         <v>45504</v>
       </c>
@@ -6032,14 +6449,29 @@
       <c r="K130">
         <v>20.5</v>
       </c>
-      <c r="L130">
-        <v>0</v>
-      </c>
-      <c r="S130" t="s">
+      <c r="L130" t="s">
+        <v>33</v>
+      </c>
+      <c r="N130">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="O130" t="s">
+        <v>33</v>
+      </c>
+      <c r="P130" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q130">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="R130">
+        <v>0.75990000000000002</v>
+      </c>
+      <c r="T130" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
         <v>45504</v>
       </c>
@@ -6067,23 +6499,26 @@
       <c r="L131">
         <v>46.6</v>
       </c>
-      <c r="N131" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O131" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P131" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q131" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S131" t="s">
+      <c r="N131" t="s">
+        <v>33</v>
+      </c>
+      <c r="O131" t="s">
+        <v>33</v>
+      </c>
+      <c r="P131" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q131" t="s">
+        <v>33</v>
+      </c>
+      <c r="R131">
+        <v>6.9400000000000003E-2</v>
+      </c>
+      <c r="T131" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
         <v>45504</v>
       </c>
@@ -6108,26 +6543,29 @@
       <c r="J132">
         <v>0.22600000000000001</v>
       </c>
-      <c r="L132">
-        <v>0</v>
-      </c>
-      <c r="N132" s="3">
+      <c r="L132" t="s">
+        <v>33</v>
+      </c>
+      <c r="N132">
         <v>0.38</v>
       </c>
-      <c r="O132" s="3">
-        <v>0.60200000000000009</v>
-      </c>
-      <c r="P132" s="3" t="s">
+      <c r="O132">
+        <v>0.60199999999999998</v>
+      </c>
+      <c r="P132" t="s">
         <v>33</v>
       </c>
       <c r="Q132">
         <v>9.9500000000000005E-2</v>
       </c>
-      <c r="S132" t="s">
+      <c r="R132">
+        <v>0.61539999999999995</v>
+      </c>
+      <c r="T132" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A133" s="1">
         <v>45518</v>
       </c>
@@ -6152,8 +6590,8 @@
       <c r="J133">
         <v>48100</v>
       </c>
-      <c r="L133">
-        <v>0</v>
+      <c r="L133" t="s">
+        <v>33</v>
       </c>
       <c r="N133">
         <v>0.59399999999999997</v>
@@ -6167,8 +6605,11 @@
       <c r="Q133" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R133">
+        <v>0.30159999999999998</v>
+      </c>
+    </row>
+    <row r="134" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A134" s="1">
         <v>45518</v>
       </c>
@@ -6190,11 +6631,11 @@
       <c r="H134">
         <v>139.6</v>
       </c>
-      <c r="J134">
-        <v>0</v>
-      </c>
-      <c r="L134">
-        <v>0</v>
+      <c r="J134" t="s">
+        <v>33</v>
+      </c>
+      <c r="L134" t="s">
+        <v>33</v>
       </c>
       <c r="N134">
         <v>8.1000000000000003E-2</v>
@@ -6208,8 +6649,11 @@
       <c r="Q134">
         <v>8.1000000000000003E-2</v>
       </c>
-    </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R134">
+        <v>0.73580000000000001</v>
+      </c>
+    </row>
+    <row r="135" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A135" s="1">
         <v>45518</v>
       </c>
@@ -6249,8 +6693,11 @@
       <c r="Q135">
         <v>0.26600000000000001</v>
       </c>
-    </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R135">
+        <v>0.3468</v>
+      </c>
+    </row>
+    <row r="136" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
         <v>45518</v>
       </c>
@@ -6275,26 +6722,29 @@
       <c r="J136">
         <v>1236</v>
       </c>
-      <c r="L136">
-        <v>0</v>
-      </c>
-      <c r="N136" s="3">
-        <v>2.5140000000000002</v>
-      </c>
-      <c r="O136" s="3">
+      <c r="L136" t="s">
+        <v>33</v>
+      </c>
+      <c r="N136">
+        <v>2.5139999999999998</v>
+      </c>
+      <c r="O136">
         <v>1.9824999999999999</v>
       </c>
-      <c r="P136" s="3" t="s">
+      <c r="P136" t="s">
         <v>33</v>
       </c>
       <c r="Q136">
         <v>0.53200000000000003</v>
       </c>
-      <c r="S136" t="s">
+      <c r="R136">
+        <v>0.60840000000000005</v>
+      </c>
+      <c r="T136" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A137" s="1">
         <v>45530</v>
       </c>
@@ -6319,8 +6769,8 @@
       <c r="J137">
         <v>1.04</v>
       </c>
-      <c r="L137">
-        <v>0</v>
+      <c r="L137" t="s">
+        <v>33</v>
       </c>
       <c r="N137">
         <v>0.34100000000000003</v>
@@ -6334,8 +6784,11 @@
       <c r="Q137">
         <v>7.8E-2</v>
       </c>
-    </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R137">
+        <v>0.24110000000000001</v>
+      </c>
+    </row>
+    <row r="138" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A138" s="1">
         <v>45530</v>
       </c>
@@ -6357,11 +6810,11 @@
       <c r="H138">
         <v>195.7</v>
       </c>
-      <c r="J138">
-        <v>0</v>
-      </c>
-      <c r="L138">
-        <v>0</v>
+      <c r="J138" t="s">
+        <v>33</v>
+      </c>
+      <c r="L138" t="s">
+        <v>33</v>
       </c>
       <c r="N138">
         <v>1.6970000000000001</v>
@@ -6375,8 +6828,11 @@
       <c r="Q138">
         <v>0.46600000000000003</v>
       </c>
-    </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R138">
+        <v>0.7167</v>
+      </c>
+    </row>
+    <row r="139" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A139" s="1">
         <v>45530</v>
       </c>
@@ -6398,11 +6854,11 @@
       <c r="H139">
         <v>52.2</v>
       </c>
-      <c r="J139">
-        <v>0</v>
-      </c>
-      <c r="L139">
-        <v>0</v>
+      <c r="J139" t="s">
+        <v>33</v>
+      </c>
+      <c r="L139" t="s">
+        <v>33</v>
       </c>
       <c r="N139">
         <v>1.0669999999999999</v>
@@ -6416,8 +6872,11 @@
       <c r="Q139">
         <v>0.40400000000000003</v>
       </c>
-    </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R139">
+        <v>0.56269999999999998</v>
+      </c>
+    </row>
+    <row r="140" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A140" s="1">
         <v>45530</v>
       </c>
@@ -6457,8 +6916,11 @@
       <c r="Q140">
         <v>0.61599999999999999</v>
       </c>
-    </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R140">
+        <v>0.58079999999999998</v>
+      </c>
+    </row>
+    <row r="141" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A141" s="1">
         <v>45549</v>
       </c>
@@ -6486,23 +6948,26 @@
       <c r="L141">
         <v>209</v>
       </c>
-      <c r="N141" s="3">
-        <v>3.266666666666667E-2</v>
-      </c>
-      <c r="O141" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P141" s="3" t="s">
+      <c r="N141">
+        <v>3.2666667000000003E-2</v>
+      </c>
+      <c r="O141" t="s">
+        <v>33</v>
+      </c>
+      <c r="P141" t="s">
         <v>33</v>
       </c>
       <c r="Q141">
-        <v>3.266666666666667E-2</v>
-      </c>
-      <c r="S141" t="s">
+        <v>3.2666667000000003E-2</v>
+      </c>
+      <c r="R141">
+        <v>0.60580000000000001</v>
+      </c>
+      <c r="T141" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A142" s="1">
         <v>45549</v>
       </c>
@@ -6542,8 +7007,11 @@
       <c r="Q142">
         <v>9.6000000000000002E-2</v>
       </c>
-    </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R142">
+        <v>0.1457</v>
+      </c>
+    </row>
+    <row r="143" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A143" s="1">
         <v>45549</v>
       </c>
@@ -6583,8 +7051,11 @@
       <c r="Q143">
         <v>8.5999999999999993E-2</v>
       </c>
-    </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R143">
+        <v>0.53520000000000001</v>
+      </c>
+    </row>
+    <row r="144" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A144" s="1">
         <v>45549</v>
       </c>
@@ -6624,8 +7095,11 @@
       <c r="Q144" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R144">
+        <v>0.68820000000000003</v>
+      </c>
+    </row>
+    <row r="145" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A145" s="1">
         <v>45562</v>
       </c>
@@ -6647,14 +7121,17 @@
       <c r="H145">
         <v>321.3</v>
       </c>
-      <c r="J145">
-        <v>0</v>
-      </c>
-      <c r="L145">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="J145" t="s">
+        <v>33</v>
+      </c>
+      <c r="L145" t="s">
+        <v>33</v>
+      </c>
+      <c r="R145">
+        <v>1.1056999999999999</v>
+      </c>
+    </row>
+    <row r="146" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A146" s="1">
         <v>45562</v>
       </c>
@@ -6671,7 +7148,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A147" s="1">
         <v>45562</v>
       </c>
@@ -6699,8 +7176,11 @@
       <c r="L147">
         <v>7.91</v>
       </c>
-    </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R147">
+        <v>0.57430000000000003</v>
+      </c>
+    </row>
+    <row r="148" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A148" s="1">
         <v>45562</v>
       </c>
@@ -6725,8 +7205,8 @@
       <c r="J148">
         <v>0.72799999999999998</v>
       </c>
-      <c r="L148">
-        <v>0</v>
+      <c r="L148" t="s">
+        <v>33</v>
       </c>
       <c r="N148" t="s">
         <v>33</v>
@@ -6740,8 +7220,11 @@
       <c r="Q148" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R148">
+        <v>0.52749999999999997</v>
+      </c>
+    </row>
+    <row r="149" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A149" s="1">
         <v>45575</v>
       </c>
@@ -6769,8 +7252,11 @@
       <c r="L149">
         <v>7.78</v>
       </c>
-    </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R149">
+        <v>0.62739999999999996</v>
+      </c>
+    </row>
+    <row r="150" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A150" s="1">
         <v>45575</v>
       </c>
@@ -6787,7 +7273,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A151" s="1">
         <v>45575</v>
       </c>
@@ -6809,14 +7295,14 @@
       <c r="H151">
         <v>142</v>
       </c>
-      <c r="J151">
-        <v>0</v>
-      </c>
-      <c r="L151">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="J151" t="s">
+        <v>33</v>
+      </c>
+      <c r="L151" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="152" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A152" s="1">
         <v>45575</v>
       </c>
@@ -6838,8 +7324,8 @@
       <c r="H152">
         <v>327.3</v>
       </c>
-      <c r="J152">
-        <v>0</v>
+      <c r="J152" t="s">
+        <v>33</v>
       </c>
       <c r="L152">
         <v>13.3</v>
@@ -6856,11 +7342,14 @@
       <c r="Q152" t="s">
         <v>33</v>
       </c>
-      <c r="S152" t="s">
+      <c r="R152">
+        <v>0.6482</v>
+      </c>
+      <c r="T152" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A153" s="1">
         <v>45490</v>
       </c>
@@ -6877,7 +7366,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A154" s="1">
         <v>45490</v>
       </c>
@@ -6894,7 +7383,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A155" s="1">
         <v>45490</v>
       </c>
@@ -6911,7 +7400,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A156" s="1">
         <v>45490</v>
       </c>
@@ -6939,8 +7428,11 @@
       <c r="L156">
         <v>28883</v>
       </c>
-    </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R156">
+        <v>0.33510000000000001</v>
+      </c>
+    </row>
+    <row r="157" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A157" s="1">
         <v>45504</v>
       </c>
@@ -6980,8 +7472,11 @@
       <c r="Q157">
         <v>1.389</v>
       </c>
-    </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R157">
+        <v>0.44090000000000001</v>
+      </c>
+    </row>
+    <row r="158" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A158" s="1">
         <v>45504</v>
       </c>
@@ -7009,8 +7504,8 @@
       <c r="K158">
         <v>904</v>
       </c>
-      <c r="L158">
-        <v>0</v>
+      <c r="L158" t="s">
+        <v>33</v>
       </c>
       <c r="N158">
         <v>1.2410000000000001</v>
@@ -7024,8 +7519,11 @@
       <c r="Q158">
         <v>0.23599999999999999</v>
       </c>
-    </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R158">
+        <v>0.50270000000000004</v>
+      </c>
+    </row>
+    <row r="159" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A159" s="1">
         <v>45504</v>
       </c>
@@ -7053,14 +7551,17 @@
       <c r="K159">
         <v>10590</v>
       </c>
-      <c r="L159">
-        <v>0</v>
-      </c>
-      <c r="S159" t="s">
+      <c r="L159" t="s">
+        <v>33</v>
+      </c>
+      <c r="R159">
+        <v>0.50270000000000004</v>
+      </c>
+      <c r="T159" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A160" s="1">
         <v>45504</v>
       </c>
@@ -7088,23 +7589,26 @@
       <c r="L160">
         <v>34938</v>
       </c>
-      <c r="N160" s="3">
-        <v>1.1113333333333333</v>
-      </c>
-      <c r="O160" s="3">
-        <v>0.89833333333333332</v>
-      </c>
-      <c r="P160" s="3" t="s">
+      <c r="N160">
+        <v>1.1113333329999999</v>
+      </c>
+      <c r="O160">
+        <v>0.89833333299999996</v>
+      </c>
+      <c r="P160" t="s">
         <v>33</v>
       </c>
       <c r="Q160">
-        <v>0.21366666666666667</v>
-      </c>
-      <c r="S160" t="s">
+        <v>0.213666667</v>
+      </c>
+      <c r="R160">
+        <v>0.31230000000000002</v>
+      </c>
+      <c r="T160" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A161" s="1">
         <v>45504</v>
       </c>
@@ -7132,23 +7636,26 @@
       <c r="L161">
         <v>1196</v>
       </c>
-      <c r="N161" s="3">
+      <c r="N161">
         <v>3.0274999999999999</v>
       </c>
-      <c r="O161" s="3">
+      <c r="O161">
         <v>2.71</v>
       </c>
-      <c r="P161" s="3" t="s">
+      <c r="P161" t="s">
         <v>33</v>
       </c>
       <c r="Q161">
         <v>0.3175</v>
       </c>
-      <c r="S161" t="s">
+      <c r="R161">
+        <v>0.1409</v>
+      </c>
+      <c r="T161" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A162" s="1">
         <v>45518</v>
       </c>
@@ -7188,8 +7695,11 @@
       <c r="Q162" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R162">
+        <v>0.31940000000000002</v>
+      </c>
+    </row>
+    <row r="163" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A163" s="1">
         <v>45518</v>
       </c>
@@ -7211,11 +7721,11 @@
       <c r="H163">
         <v>114.2</v>
       </c>
-      <c r="J163">
-        <v>0</v>
-      </c>
-      <c r="L163">
-        <v>0</v>
+      <c r="J163" t="s">
+        <v>33</v>
+      </c>
+      <c r="L163" t="s">
+        <v>33</v>
       </c>
       <c r="N163" t="s">
         <v>33</v>
@@ -7229,8 +7739,11 @@
       <c r="Q163" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R163">
+        <v>0.20399999999999999</v>
+      </c>
+    </row>
+    <row r="164" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A164" s="1">
         <v>45518</v>
       </c>
@@ -7252,8 +7765,8 @@
       <c r="H164">
         <v>324.39999999999998</v>
       </c>
-      <c r="J164">
-        <v>0</v>
+      <c r="J164" t="s">
+        <v>33</v>
       </c>
       <c r="L164">
         <v>3910000</v>
@@ -7273,8 +7786,11 @@
       <c r="Q164">
         <v>0.77</v>
       </c>
-    </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R164">
+        <v>0.1016</v>
+      </c>
+    </row>
+    <row r="165" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A165" s="1">
         <v>45518</v>
       </c>
@@ -7296,8 +7812,8 @@
       <c r="H165">
         <v>206.2</v>
       </c>
-      <c r="J165">
-        <v>0</v>
+      <c r="J165" t="s">
+        <v>33</v>
       </c>
       <c r="L165">
         <v>1990000</v>
@@ -7305,23 +7821,26 @@
       <c r="M165">
         <v>652</v>
       </c>
-      <c r="N165" s="3">
-        <v>0.53799999999999992</v>
-      </c>
-      <c r="O165" s="3">
-        <v>0.44833333333333331</v>
-      </c>
-      <c r="P165" s="3" t="s">
+      <c r="N165">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="O165">
+        <v>0.448333333</v>
+      </c>
+      <c r="P165" t="s">
         <v>33</v>
       </c>
       <c r="Q165">
-        <v>8.9666666666666672E-2</v>
-      </c>
-      <c r="S165" t="s">
+        <v>8.9666667000000005E-2</v>
+      </c>
+      <c r="R165">
+        <v>0.33760000000000001</v>
+      </c>
+      <c r="T165" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A166" s="1">
         <v>45530</v>
       </c>
@@ -7361,8 +7880,11 @@
       <c r="Q166">
         <v>0.81799999999999995</v>
       </c>
-    </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R166">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="167" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A167" s="1">
         <v>45530</v>
       </c>
@@ -7390,23 +7912,26 @@
       <c r="L167">
         <v>1202</v>
       </c>
-      <c r="N167" s="3">
+      <c r="N167">
         <v>6.5780000000000003</v>
       </c>
-      <c r="O167" s="3">
-        <v>4.7316666666666665</v>
-      </c>
-      <c r="P167" s="3" t="s">
+      <c r="O167">
+        <v>4.7316666669999998</v>
+      </c>
+      <c r="P167" t="s">
         <v>33</v>
       </c>
       <c r="Q167">
         <v>1.8460000000000001</v>
       </c>
-      <c r="S167" t="s">
+      <c r="R167">
+        <v>0.46879999999999999</v>
+      </c>
+      <c r="T167" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A168" s="1">
         <v>45530</v>
       </c>
@@ -7434,8 +7959,11 @@
       <c r="Q168">
         <v>0.42599999999999999</v>
       </c>
-    </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R168">
+        <v>0.35049999999999998</v>
+      </c>
+    </row>
+    <row r="169" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A169" s="1">
         <v>45530</v>
       </c>
@@ -7463,8 +7991,11 @@
       <c r="Q169">
         <v>0.55300000000000005</v>
       </c>
-    </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R169">
+        <v>0.22550000000000001</v>
+      </c>
+    </row>
+    <row r="170" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A170" s="1">
         <v>45549</v>
       </c>
@@ -7480,23 +8011,26 @@
       <c r="E170" t="s">
         <v>21</v>
       </c>
-      <c r="N170" s="3">
-        <v>7.2333333333333319E-2</v>
-      </c>
-      <c r="O170" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P170" s="3" t="s">
+      <c r="N170">
+        <v>7.2333333E-2</v>
+      </c>
+      <c r="O170" t="s">
+        <v>33</v>
+      </c>
+      <c r="P170" t="s">
         <v>33</v>
       </c>
       <c r="Q170">
-        <v>7.2333333333333319E-2</v>
-      </c>
-      <c r="S170" t="s">
+        <v>7.2333333E-2</v>
+      </c>
+      <c r="R170">
+        <v>0.34310000000000002</v>
+      </c>
+      <c r="T170" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A171" s="1">
         <v>45549</v>
       </c>
@@ -7524,8 +8058,11 @@
       <c r="Q171">
         <v>0.158</v>
       </c>
-    </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R171">
+        <v>0.30420000000000003</v>
+      </c>
+    </row>
+    <row r="172" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A172" s="1">
         <v>45549</v>
       </c>
@@ -7553,8 +8090,11 @@
       <c r="Q172">
         <v>6.6000000000000003E-2</v>
       </c>
-    </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="R172">
+        <v>0.82169999999999999</v>
+      </c>
+    </row>
+    <row r="173" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A173" s="1">
         <v>45549</v>
       </c>
@@ -7581,9 +8121,295 @@
       </c>
       <c r="Q173">
         <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="R173">
+        <v>0.33560000000000001</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D264E2-9F84-5F4C-83B6-1DE69BA5700F}">
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>46065</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="4" spans="1:7" ht="88" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="8"/>
+      <c r="B11" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="8"/>
+      <c r="B12" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="8"/>
+      <c r="B13" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="8"/>
+      <c r="B14" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="8"/>
+      <c r="B15" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A21" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A23" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A24" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="8"/>
+      <c r="B29" s="6"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="8"/>
+      <c r="B30" s="6"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="12"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="8"/>
+      <c r="B32" s="6"/>
+    </row>
+    <row r="33" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A33" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="68" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A35" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="8"/>
+      <c r="B36" s="7"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="8"/>
+      <c r="B37" s="7"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="8"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="8"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="8"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="8"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="8"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:G4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Cleared environment, cleaning code
</commit_message>
<xml_diff>
--- a/data/qPCR_Anatoxins_forGoel.xlsx
+++ b/data/qPCR_Anatoxins_forGoel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jld/Documents/Github/River_HAB_Modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB37516-E68D-AF47-B906-2CF2A7686525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34604F4-1CB4-5244-9525-337BB502CB94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1600" yWindow="760" windowWidth="27640" windowHeight="18880" activeTab="1" xr2:uid="{EF90CB1A-CFB2-4A4B-95FD-9B0D7CA467ED}"/>
+    <workbookView xWindow="1600" yWindow="760" windowWidth="27640" windowHeight="18880" xr2:uid="{EF90CB1A-CFB2-4A4B-95FD-9B0D7CA467ED}"/>
   </bookViews>
   <sheets>
     <sheet name="qPCR_Anatoxins" sheetId="1" r:id="rId1"/>
@@ -760,15 +760,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -789,6 +780,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -7498,7 +7498,7 @@
       <c r="H158">
         <v>125.1</v>
       </c>
-      <c r="J158">
+      <c r="J158" s="2">
         <v>124000000</v>
       </c>
       <c r="K158">
@@ -7545,7 +7545,7 @@
       <c r="H159">
         <v>35.200000000000003</v>
       </c>
-      <c r="J159">
+      <c r="J159" s="2">
         <v>1.1200000000000001</v>
       </c>
       <c r="K159">
@@ -8141,31 +8141,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
+      <c r="A2" s="11">
         <v>46065</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
     </row>
     <row r="4" spans="1:7" ht="88" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -8176,233 +8176,233 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="8"/>
+      <c r="B7" s="5"/>
     </row>
     <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="8"/>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="4" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="8"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="8"/>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="4" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="8"/>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="7" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="4" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="51" x14ac:dyDescent="0.2">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="4" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="7" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="4" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="4" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="8"/>
-      <c r="B29" s="6"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="3"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="8"/>
-      <c r="B30" s="6"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="3"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="12"/>
+      <c r="B31" s="9"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="8"/>
-      <c r="B32" s="6"/>
+      <c r="A32" s="5"/>
+      <c r="B32" s="3"/>
     </row>
     <row r="33" spans="1:2" ht="51" x14ac:dyDescent="0.2">
-      <c r="A33" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="10" t="s">
+      <c r="A33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="68" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34" s="10" t="s">
+      <c r="A34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="8"/>
-      <c r="B36" s="7"/>
+      <c r="A36" s="5"/>
+      <c r="B36" s="4"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="8"/>
-      <c r="B37" s="7"/>
+      <c r="A37" s="5"/>
+      <c r="B37" s="4"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="8"/>
+      <c r="A38" s="5"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="8"/>
+      <c r="A39" s="5"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="8"/>
+      <c r="A40" s="5"/>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="8"/>
+      <c r="A41" s="5"/>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="8"/>
+      <c r="A42" s="5"/>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="8"/>
+      <c r="A43" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Cleaning data files. Cleaning old commented-out code. Wrote new code to make sure both original samples and rerun samples for qPCR were all getting plotted
</commit_message>
<xml_diff>
--- a/data/qPCR_Anatoxins_forGoel.xlsx
+++ b/data/qPCR_Anatoxins_forGoel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jld/Documents/Github/River_HAB_Modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34604F4-1CB4-5244-9525-337BB502CB94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA3717B-3BDA-DE46-B320-553EB056FCDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1600" yWindow="760" windowWidth="27640" windowHeight="18880" xr2:uid="{EF90CB1A-CFB2-4A4B-95FD-9B0D7CA467ED}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="77">
   <si>
     <t>date</t>
   </si>
@@ -141,9 +141,6 @@
     <t>Original file said 5404 for ana_C/ul, but newer file from 1/2026 says 43.9</t>
   </si>
   <si>
-    <t>PCR duplicate</t>
-  </si>
-  <si>
     <t>qPCR reruns for 2024 performed on the same samples as before</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>Indicates whether mat material for qPCR analysis was present for collection in the field</t>
   </si>
   <si>
-    <t>sample_rerun</t>
-  </si>
-  <si>
     <t>Vial ID # of samples (mailed in Oct. 2025)</t>
   </si>
   <si>
@@ -257,12 +251,45 @@
   <si>
     <t>No collected sample</t>
   </si>
+  <si>
+    <t>nd</t>
+  </si>
+  <si>
+    <t>PCR duplicate, no DNA_conc for rerun</t>
+  </si>
+  <si>
+    <t>No given DNA_conc for rerun</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">Important note: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>In 2024, some original samples were rerun using qPCR. Each rerun was given a new ID by adding “.1” to the original sample number (e.g. sample 34 became 34.1).
+Because the reruns used the same samples, previously measured gene values were reused as needed. The reruns tested only one gene (anaC or nif) per sample. The value for the gene that was not retested was copied from the original results into the rerun column (e.g. if sample 34 was rerun for anaC only, the original nif value (34) was copied into the rerun entry (34.1).
+No rerun in 2024 tested both genes for the same sample. All reruns in 2023 were performed on separately collected duplicates, rather than the single originally tested sample.</t>
+    </r>
+  </si>
+  <si>
+    <t>Non-detect</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -405,6 +432,12 @@
     <font>
       <b/>
       <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos"/>
     </font>
@@ -1167,12 +1200,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA4CAA07-9486-4548-BA57-E25BF6238077}">
   <dimension ref="A1:T173"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1227,7 +1254,7 @@
         <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="S1" t="s">
         <v>17</v>
@@ -1973,10 +2000,10 @@
         <v>75.3</v>
       </c>
       <c r="K26" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M26" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N26">
         <v>8.1000000000000003E-2</v>
@@ -2026,13 +2053,13 @@
         <v>20</v>
       </c>
       <c r="K27" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L27" t="s">
         <v>20</v>
       </c>
       <c r="M27" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N27">
         <v>0.313</v>
@@ -2111,13 +2138,13 @@
         <v>20</v>
       </c>
       <c r="K29" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L29" t="s">
         <v>20</v>
       </c>
       <c r="M29" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N29">
         <v>0.17799999999999999</v>
@@ -2173,7 +2200,7 @@
         <v>20</v>
       </c>
       <c r="M30" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N30">
         <v>2.758</v>
@@ -2223,13 +2250,13 @@
         <v>20</v>
       </c>
       <c r="K31" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L31" t="s">
         <v>20</v>
       </c>
       <c r="M31" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N31">
         <v>1.8879999999999999</v>
@@ -2323,13 +2350,13 @@
         <v>20</v>
       </c>
       <c r="K33" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L33" t="s">
         <v>20</v>
       </c>
       <c r="M33" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N33">
         <v>0.36430000000000001</v>
@@ -2373,7 +2400,7 @@
         <v>141</v>
       </c>
       <c r="L34" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N34">
         <v>1.9319999999999999</v>
@@ -2423,13 +2450,13 @@
         <v>20</v>
       </c>
       <c r="K35" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L35" t="s">
         <v>20</v>
       </c>
       <c r="M35" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N35">
         <v>6.6467000000000001</v>
@@ -2505,7 +2532,7 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="K37" t="s">
         <v>20</v>
@@ -2561,7 +2588,7 @@
         <v>3.37</v>
       </c>
       <c r="L38" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N38">
         <v>17.29</v>
@@ -2611,13 +2638,13 @@
         <v>20</v>
       </c>
       <c r="K39" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L39" t="s">
         <v>20</v>
       </c>
       <c r="M39" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N39">
         <v>7.3623000000000003</v>
@@ -2661,7 +2688,7 @@
         <v>7161</v>
       </c>
       <c r="M40" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N40">
         <v>99.066000000000003</v>
@@ -2761,10 +2788,10 @@
         <v>49</v>
       </c>
       <c r="J42" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L42" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="T42" t="s">
         <v>30</v>
@@ -2859,7 +2886,7 @@
         <v>68</v>
       </c>
       <c r="J46" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="K46">
         <v>4930</v>
@@ -2909,10 +2936,10 @@
         <v>19</v>
       </c>
       <c r="J47" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L47" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="T47" t="s">
         <v>32</v>
@@ -3061,7 +3088,7 @@
         <v>85.1</v>
       </c>
       <c r="L51" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N51">
         <v>18.032</v>
@@ -3105,7 +3132,7 @@
         <v>43.9</v>
       </c>
       <c r="L52" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N52">
         <v>25.83</v>
@@ -3252,7 +3279,7 @@
         <v>20</v>
       </c>
       <c r="M55" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N55">
         <v>9.8970000000000002</v>
@@ -3270,7 +3297,7 @@
         <v>0.61299999999999999</v>
       </c>
       <c r="T55" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.2">
@@ -3305,13 +3332,13 @@
         <v>5404</v>
       </c>
       <c r="K56" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L56" t="s">
         <v>20</v>
       </c>
       <c r="M56" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N56">
         <v>19.989999999999998</v>
@@ -3361,7 +3388,7 @@
         <v>57.3</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="K57" s="2">
         <v>20904</v>
@@ -3538,13 +3565,13 @@
         <v>103</v>
       </c>
       <c r="K60" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L60" t="s">
         <v>20</v>
       </c>
       <c r="M60" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N60">
         <v>12.81</v>
@@ -3591,7 +3618,7 @@
         <v>96.1</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="K61" s="2">
         <v>22269</v>
@@ -4038,7 +4065,7 @@
         <v>58.1</v>
       </c>
       <c r="K70" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M70">
         <v>870</v>
@@ -4140,7 +4167,7 @@
         <v>84.6</v>
       </c>
       <c r="K73" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M73">
         <v>1299</v>
@@ -4272,10 +4299,10 @@
         <v>65.2</v>
       </c>
       <c r="K76" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M76" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N76">
         <v>8.7999999999999995E-2</v>
@@ -4316,10 +4343,10 @@
         <v>59.9</v>
       </c>
       <c r="K77" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M77" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N77">
         <v>0.77800000000000002</v>
@@ -4392,10 +4419,10 @@
         <v>159</v>
       </c>
       <c r="K79" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M79" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N79">
         <v>5.0190000000000001</v>
@@ -4436,10 +4463,10 @@
         <v>80.7</v>
       </c>
       <c r="K80" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M80" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N80">
         <v>0.76300000000000001</v>
@@ -4530,7 +4557,7 @@
         <v>12.8</v>
       </c>
       <c r="M82" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N82">
         <v>3.6920000000000002</v>
@@ -4571,7 +4598,7 @@
         <v>132</v>
       </c>
       <c r="K83" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M83">
         <v>29532</v>
@@ -4659,10 +4686,10 @@
         <v>76.2</v>
       </c>
       <c r="K85" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M85" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N85">
         <v>38.588000000000001</v>
@@ -4706,7 +4733,7 @@
         <v>37339</v>
       </c>
       <c r="M86" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N86">
         <v>7.1319999999999997</v>
@@ -4747,10 +4774,10 @@
         <v>58.6</v>
       </c>
       <c r="K87" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M87" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N87">
         <v>51.351999999999997</v>
@@ -4794,7 +4821,7 @@
         <v>16234</v>
       </c>
       <c r="M88" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N88">
         <v>24.847300000000001</v>
@@ -4835,10 +4862,10 @@
         <v>47.9</v>
       </c>
       <c r="K89" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M89" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N89">
         <v>25.082000000000001</v>
@@ -4879,10 +4906,10 @@
         <v>188.1</v>
       </c>
       <c r="K90" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M90" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N90">
         <v>36.5015</v>
@@ -5011,10 +5038,10 @@
         <v>28.2</v>
       </c>
       <c r="K93" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M93" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N93">
         <v>32.741</v>
@@ -5055,10 +5082,10 @@
         <v>151.80000000000001</v>
       </c>
       <c r="K94" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M94" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N94">
         <v>15.971500000000001</v>
@@ -5178,10 +5205,10 @@
         <v>63.7</v>
       </c>
       <c r="K97" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="M97" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.2">
@@ -5808,7 +5835,7 @@
         <v>21</v>
       </c>
       <c r="T115" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="116" spans="1:20" x14ac:dyDescent="0.2">
@@ -5839,6 +5866,9 @@
       <c r="L116">
         <v>497</v>
       </c>
+      <c r="T116" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="117" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
@@ -5910,7 +5940,7 @@
         <v>5.31</v>
       </c>
       <c r="L118" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N118" t="s">
         <v>33</v>
@@ -5960,7 +5990,7 @@
         <v>0.3528</v>
       </c>
       <c r="T119" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="120" spans="1:20" x14ac:dyDescent="0.2">
@@ -5986,10 +6016,10 @@
         <v>384.8</v>
       </c>
       <c r="J120" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L120" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N120" t="s">
         <v>33</v>
@@ -6074,7 +6104,7 @@
         <v>60.3</v>
       </c>
       <c r="J122" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L122">
         <v>17562</v>
@@ -6158,6 +6188,9 @@
       <c r="F124">
         <v>12</v>
       </c>
+      <c r="G124">
+        <v>12.1</v>
+      </c>
       <c r="H124">
         <v>208.3</v>
       </c>
@@ -6168,7 +6201,10 @@
         <v>271</v>
       </c>
       <c r="L124" t="s">
-        <v>33</v>
+        <v>72</v>
+      </c>
+      <c r="M124" t="s">
+        <v>72</v>
       </c>
       <c r="N124" t="s">
         <v>33</v>
@@ -6186,7 +6222,7 @@
         <v>0.6139</v>
       </c>
       <c r="T124" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
     </row>
     <row r="125" spans="1:20" x14ac:dyDescent="0.2">
@@ -6208,6 +6244,9 @@
       <c r="F125">
         <v>13</v>
       </c>
+      <c r="G125">
+        <v>13.1</v>
+      </c>
       <c r="H125">
         <v>223.4</v>
       </c>
@@ -6220,6 +6259,9 @@
       <c r="L125">
         <v>30</v>
       </c>
+      <c r="M125">
+        <v>30</v>
+      </c>
       <c r="N125" t="s">
         <v>33</v>
       </c>
@@ -6236,7 +6278,7 @@
         <v>0.6139</v>
       </c>
       <c r="T125" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="126" spans="1:20" x14ac:dyDescent="0.2">
@@ -6265,7 +6307,7 @@
         <v>22.1</v>
       </c>
       <c r="L126" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N126" t="s">
         <v>33</v>
@@ -6327,7 +6369,7 @@
         <v>0.56040000000000001</v>
       </c>
       <c r="T127" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="128" spans="1:20" x14ac:dyDescent="0.2">
@@ -6393,17 +6435,23 @@
       <c r="F129">
         <v>32</v>
       </c>
+      <c r="G129">
+        <v>32.1</v>
+      </c>
       <c r="H129">
         <v>347</v>
       </c>
       <c r="J129" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="K129">
         <v>10.67</v>
       </c>
       <c r="L129" t="s">
-        <v>33</v>
+        <v>72</v>
+      </c>
+      <c r="M129" t="s">
+        <v>72</v>
       </c>
       <c r="N129">
         <v>5.8999999999999997E-2</v>
@@ -6419,6 +6467,9 @@
       </c>
       <c r="R129">
         <v>0.75990000000000002</v>
+      </c>
+      <c r="T129" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="130" spans="1:20" x14ac:dyDescent="0.2">
@@ -6440,6 +6491,9 @@
       <c r="F130">
         <v>33</v>
       </c>
+      <c r="G130">
+        <v>33.1</v>
+      </c>
       <c r="H130">
         <v>294.3</v>
       </c>
@@ -6450,7 +6504,10 @@
         <v>20.5</v>
       </c>
       <c r="L130" t="s">
-        <v>33</v>
+        <v>72</v>
+      </c>
+      <c r="M130" t="s">
+        <v>72</v>
       </c>
       <c r="N130">
         <v>5.8999999999999997E-2</v>
@@ -6468,7 +6525,7 @@
         <v>0.75990000000000002</v>
       </c>
       <c r="T130" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="131" spans="1:20" x14ac:dyDescent="0.2">
@@ -6515,7 +6572,7 @@
         <v>6.9400000000000003E-2</v>
       </c>
       <c r="T131" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="132" spans="1:20" x14ac:dyDescent="0.2">
@@ -6544,7 +6601,7 @@
         <v>0.22600000000000001</v>
       </c>
       <c r="L132" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N132">
         <v>0.38</v>
@@ -6562,7 +6619,7 @@
         <v>0.61539999999999995</v>
       </c>
       <c r="T132" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="133" spans="1:20" x14ac:dyDescent="0.2">
@@ -6591,7 +6648,7 @@
         <v>48100</v>
       </c>
       <c r="L133" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N133">
         <v>0.59399999999999997</v>
@@ -6632,10 +6689,10 @@
         <v>139.6</v>
       </c>
       <c r="J134" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L134" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N134">
         <v>8.1000000000000003E-2</v>
@@ -6723,7 +6780,7 @@
         <v>1236</v>
       </c>
       <c r="L136" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N136">
         <v>2.5139999999999998</v>
@@ -6741,7 +6798,7 @@
         <v>0.60840000000000005</v>
       </c>
       <c r="T136" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="137" spans="1:20" x14ac:dyDescent="0.2">
@@ -6770,7 +6827,7 @@
         <v>1.04</v>
       </c>
       <c r="L137" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N137">
         <v>0.34100000000000003</v>
@@ -6811,10 +6868,10 @@
         <v>195.7</v>
       </c>
       <c r="J138" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L138" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N138">
         <v>1.6970000000000001</v>
@@ -6855,10 +6912,10 @@
         <v>52.2</v>
       </c>
       <c r="J139" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L139" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N139">
         <v>1.0669999999999999</v>
@@ -6964,7 +7021,7 @@
         <v>0.60580000000000001</v>
       </c>
       <c r="T141" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="142" spans="1:20" x14ac:dyDescent="0.2">
@@ -7122,10 +7179,10 @@
         <v>321.3</v>
       </c>
       <c r="J145" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L145" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="R145">
         <v>1.1056999999999999</v>
@@ -7206,7 +7263,7 @@
         <v>0.72799999999999998</v>
       </c>
       <c r="L148" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N148" t="s">
         <v>33</v>
@@ -7296,10 +7353,10 @@
         <v>142</v>
       </c>
       <c r="J151" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L151" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
     </row>
     <row r="152" spans="1:20" x14ac:dyDescent="0.2">
@@ -7325,7 +7382,7 @@
         <v>327.3</v>
       </c>
       <c r="J152" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L152">
         <v>13.3</v>
@@ -7346,7 +7403,7 @@
         <v>0.6482</v>
       </c>
       <c r="T152" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="153" spans="1:20" x14ac:dyDescent="0.2">
@@ -7495,17 +7552,23 @@
       <c r="F158">
         <v>34</v>
       </c>
+      <c r="G158">
+        <v>34.1</v>
+      </c>
       <c r="H158">
         <v>125.1</v>
       </c>
       <c r="J158" s="2">
         <v>124000000</v>
       </c>
-      <c r="K158">
+      <c r="K158" s="2">
         <v>904</v>
       </c>
       <c r="L158" t="s">
-        <v>33</v>
+        <v>72</v>
+      </c>
+      <c r="M158" t="s">
+        <v>72</v>
       </c>
       <c r="N158">
         <v>1.2410000000000001</v>
@@ -7521,6 +7584,9 @@
       </c>
       <c r="R158">
         <v>0.50270000000000004</v>
+      </c>
+      <c r="T158" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="159" spans="1:20" x14ac:dyDescent="0.2">
@@ -7542,23 +7608,29 @@
       <c r="F159">
         <v>35</v>
       </c>
+      <c r="G159">
+        <v>35.1</v>
+      </c>
       <c r="H159">
         <v>35.200000000000003</v>
       </c>
       <c r="J159" s="2">
         <v>1.1200000000000001</v>
       </c>
-      <c r="K159">
+      <c r="K159" s="2">
         <v>10590</v>
       </c>
       <c r="L159" t="s">
-        <v>33</v>
+        <v>72</v>
+      </c>
+      <c r="M159" t="s">
+        <v>72</v>
       </c>
       <c r="R159">
         <v>0.50270000000000004</v>
       </c>
       <c r="T159" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="160" spans="1:20" x14ac:dyDescent="0.2">
@@ -7605,7 +7677,7 @@
         <v>0.31230000000000002</v>
       </c>
       <c r="T160" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="161" spans="1:20" x14ac:dyDescent="0.2">
@@ -7652,7 +7724,7 @@
         <v>0.1409</v>
       </c>
       <c r="T161" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="162" spans="1:20" x14ac:dyDescent="0.2">
@@ -7722,10 +7794,10 @@
         <v>114.2</v>
       </c>
       <c r="J163" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="L163" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="N163" t="s">
         <v>33</v>
@@ -7762,16 +7834,22 @@
       <c r="F164">
         <v>45</v>
       </c>
+      <c r="G164">
+        <v>45.1</v>
+      </c>
       <c r="H164">
         <v>324.39999999999998</v>
       </c>
       <c r="J164" t="s">
-        <v>33</v>
-      </c>
-      <c r="L164">
+        <v>72</v>
+      </c>
+      <c r="K164" t="s">
+        <v>72</v>
+      </c>
+      <c r="L164" s="2">
         <v>3910000</v>
       </c>
-      <c r="M164">
+      <c r="M164" s="2">
         <v>8489</v>
       </c>
       <c r="N164">
@@ -7788,6 +7866,9 @@
       </c>
       <c r="R164">
         <v>0.1016</v>
+      </c>
+      <c r="T164" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="165" spans="1:20" x14ac:dyDescent="0.2">
@@ -7809,16 +7890,22 @@
       <c r="F165">
         <v>39</v>
       </c>
+      <c r="G165">
+        <v>39.1</v>
+      </c>
       <c r="H165">
         <v>206.2</v>
       </c>
       <c r="J165" t="s">
-        <v>33</v>
-      </c>
-      <c r="L165">
+        <v>72</v>
+      </c>
+      <c r="K165" t="s">
+        <v>72</v>
+      </c>
+      <c r="L165" s="2">
         <v>1990000</v>
       </c>
-      <c r="M165">
+      <c r="M165" s="2">
         <v>652</v>
       </c>
       <c r="N165">
@@ -7837,7 +7924,7 @@
         <v>0.33760000000000001</v>
       </c>
       <c r="T165" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="166" spans="1:20" x14ac:dyDescent="0.2">
@@ -7928,7 +8015,7 @@
         <v>0.46879999999999999</v>
       </c>
       <c r="T167" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="168" spans="1:20" x14ac:dyDescent="0.2">
@@ -8027,7 +8114,7 @@
         <v>0.34310000000000002</v>
       </c>
       <c r="T170" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="171" spans="1:20" x14ac:dyDescent="0.2">
@@ -8133,7 +8220,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D264E2-9F84-5F4C-83B6-1DE69BA5700F}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.83203125" bestFit="1" customWidth="1"/>
@@ -8142,7 +8229,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -8158,7 +8245,7 @@
     </row>
     <row r="4" spans="1:7" ht="88" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -8167,230 +8254,243 @@
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+    <row r="5" spans="1:7" ht="137" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="5"/>
+    </row>
+    <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="5"/>
-    </row>
-    <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="5"/>
       <c r="B11" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="4" t="s">
+    <row r="18" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="51" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B21" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A21" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A22" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="5"/>
-      <c r="B29" s="3"/>
+      <c r="B29" s="4" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="5"/>
       <c r="B30" s="3"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="5"/>
+      <c r="B31" s="3"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32" s="9"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="5"/>
+      <c r="B33" s="3"/>
+    </row>
+    <row r="34" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="68" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="9"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="5"/>
-      <c r="B32" s="3"/>
-    </row>
-    <row r="33" spans="1:2" ht="51" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="7" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" ht="68" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34" s="7" t="s">
+      <c r="B37" s="4" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="5"/>
-      <c r="B36" s="4"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="5"/>
-      <c r="B37" s="4"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="5"/>
+      <c r="B38" s="4"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="5"/>
+      <c r="B39" s="4"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="5"/>
@@ -8404,11 +8504,18 @@
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="5"/>
     </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="5"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>